<commit_message>
fix: contract item semantic duplicates v52.48.5.44.8.3
</commit_message>
<xml_diff>
--- a/public/templates/주간업무총괄.xlsx
+++ b/public/templates/주간업무총괄.xlsx
@@ -3,8 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21328"/>
   <workbookPr defaultThemeVersion="166925"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\서재형\Desktop\new\public\templates\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74CFD619-54E1-4582-AA68-CD8D7C4FC245}" xr6:coauthVersionLast="41" xr6:coauthVersionMax="41" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F4E6143A-B7CB-4042-8A64-B22D5BBF99DC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F4E6143A-B7CB-4042-8A64-B22D5BBF99DC}"/>
   </bookViews>
   <sheets>
     <sheet name="주간업무총괄" sheetId="1" r:id="rId1"/>
@@ -414,98 +420,98 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="255"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" shrinkToFit="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -554,7 +560,7 @@
               <a:picLocks noChangeAspect="1"/>
               <a:extLst>
                 <a:ext uri="{84589F7E-364E-4C9E-8A38-B11213B215E9}">
-                  <a14:cameraTool cellRange="$H$58:$N$60" spid="_x0000_s1030"/>
+                  <a14:cameraTool cellRange="$H$58:$N$60" spid="_x0000_s1031"/>
                 </a:ext>
               </a:extLst>
             </xdr:cNvPicPr>
@@ -897,727 +903,792 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="8" t="s">
+      <c r="B1" s="32"/>
+      <c r="C1" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="30" t="s">
         <v>17</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="3" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="A2" s="32"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="30"/>
+      <c r="E2" s="31"/>
+      <c r="F2" s="31"/>
     </row>
     <row r="3" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="4"/>
-      <c r="F3" s="4"/>
+      <c r="A3" s="32"/>
+      <c r="B3" s="32"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="30"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
     </row>
     <row r="4" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="10"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
+      <c r="A4" s="32"/>
+      <c r="B4" s="32"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="30"/>
+      <c r="E4" s="31"/>
+      <c r="F4" s="31"/>
     </row>
     <row r="5" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="3" t="s">
+      <c r="A5" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
+      <c r="D5" s="29"/>
+      <c r="E5" s="29"/>
+      <c r="F5" s="29"/>
     </row>
     <row r="6" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
+      <c r="A6" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="C6" s="13" t="s">
+      <c r="C6" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="15"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="24"/>
+      <c r="F6" s="25"/>
     </row>
     <row r="7" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="16"/>
-      <c r="D7" s="17"/>
-      <c r="E7" s="17"/>
-      <c r="F7" s="18"/>
+      <c r="A7" s="29"/>
+      <c r="B7" s="29"/>
+      <c r="C7" s="14"/>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="16"/>
     </row>
     <row r="8" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="19" t="s">
+      <c r="A8" s="29"/>
+      <c r="B8" s="29"/>
+      <c r="C8" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="21"/>
+      <c r="D8" s="27"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="28"/>
     </row>
     <row r="9" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="22"/>
-      <c r="D9" s="23"/>
-      <c r="E9" s="23"/>
-      <c r="F9" s="24"/>
+      <c r="A9" s="29"/>
+      <c r="B9" s="29"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="10"/>
+      <c r="E9" s="10"/>
+      <c r="F9" s="11"/>
     </row>
     <row r="10" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2" t="s">
+      <c r="A10" s="29"/>
+      <c r="B10" s="29" t="s">
         <v>5</v>
       </c>
-      <c r="C10" s="13" t="s">
+      <c r="C10" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="15"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="25"/>
     </row>
     <row r="11" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="16"/>
-      <c r="D11" s="17"/>
-      <c r="E11" s="17"/>
-      <c r="F11" s="18"/>
+      <c r="A11" s="29"/>
+      <c r="B11" s="29"/>
+      <c r="C11" s="14"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="15"/>
+      <c r="F11" s="16"/>
     </row>
     <row r="12" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="19" t="s">
+      <c r="A12" s="29"/>
+      <c r="B12" s="29"/>
+      <c r="C12" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="21"/>
+      <c r="D12" s="27"/>
+      <c r="E12" s="27"/>
+      <c r="F12" s="28"/>
     </row>
     <row r="13" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="22"/>
-      <c r="D13" s="23"/>
-      <c r="E13" s="23"/>
-      <c r="F13" s="24"/>
+      <c r="A13" s="29"/>
+      <c r="B13" s="29"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="10"/>
+      <c r="E13" s="10"/>
+      <c r="F13" s="11"/>
     </row>
     <row r="14" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2" t="s">
+      <c r="A14" s="29"/>
+      <c r="B14" s="29" t="s">
         <v>6</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="C14" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="15"/>
+      <c r="D14" s="24"/>
+      <c r="E14" s="24"/>
+      <c r="F14" s="25"/>
     </row>
     <row r="15" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="16"/>
-      <c r="D15" s="17"/>
-      <c r="E15" s="17"/>
-      <c r="F15" s="18"/>
+      <c r="A15" s="29"/>
+      <c r="B15" s="29"/>
+      <c r="C15" s="14"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="16"/>
     </row>
     <row r="16" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="19" t="s">
+      <c r="A16" s="29"/>
+      <c r="B16" s="29"/>
+      <c r="C16" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="21"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="28"/>
     </row>
     <row r="17" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="23"/>
-      <c r="E17" s="23"/>
-      <c r="F17" s="24"/>
+      <c r="A17" s="29"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="10"/>
+      <c r="E17" s="10"/>
+      <c r="F17" s="11"/>
     </row>
     <row r="18" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2" t="s">
+      <c r="A18" s="29"/>
+      <c r="B18" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="C18" s="13" t="s">
+      <c r="C18" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="15"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="25"/>
     </row>
     <row r="19" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="17"/>
-      <c r="F19" s="18"/>
+      <c r="A19" s="29"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="15"/>
+      <c r="E19" s="15"/>
+      <c r="F19" s="16"/>
     </row>
     <row r="20" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
-      <c r="C20" s="19" t="s">
+      <c r="A20" s="29"/>
+      <c r="B20" s="29"/>
+      <c r="C20" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D20" s="20"/>
-      <c r="E20" s="20"/>
-      <c r="F20" s="21"/>
+      <c r="D20" s="27"/>
+      <c r="E20" s="27"/>
+      <c r="F20" s="28"/>
     </row>
     <row r="21" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="22"/>
-      <c r="D21" s="23"/>
-      <c r="E21" s="23"/>
-      <c r="F21" s="24"/>
+      <c r="A21" s="29"/>
+      <c r="B21" s="29"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="10"/>
+      <c r="E21" s="10"/>
+      <c r="F21" s="11"/>
     </row>
     <row r="22" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2" t="s">
+      <c r="A22" s="29"/>
+      <c r="B22" s="29" t="s">
         <v>8</v>
       </c>
-      <c r="C22" s="13" t="s">
+      <c r="C22" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D22" s="14"/>
-      <c r="E22" s="14"/>
-      <c r="F22" s="15"/>
+      <c r="D22" s="24"/>
+      <c r="E22" s="24"/>
+      <c r="F22" s="25"/>
     </row>
     <row r="23" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
-      <c r="C23" s="16"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
-      <c r="F23" s="18"/>
+      <c r="A23" s="29"/>
+      <c r="B23" s="29"/>
+      <c r="C23" s="14"/>
+      <c r="D23" s="15"/>
+      <c r="E23" s="15"/>
+      <c r="F23" s="16"/>
     </row>
     <row r="24" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
-      <c r="C24" s="19" t="s">
+      <c r="A24" s="29"/>
+      <c r="B24" s="29"/>
+      <c r="C24" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="20"/>
-      <c r="E24" s="20"/>
-      <c r="F24" s="21"/>
+      <c r="D24" s="27"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="28"/>
     </row>
     <row r="25" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
-      <c r="C25" s="22"/>
-      <c r="D25" s="23"/>
-      <c r="E25" s="23"/>
-      <c r="F25" s="24"/>
+      <c r="A25" s="29"/>
+      <c r="B25" s="29"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="10"/>
+      <c r="E25" s="10"/>
+      <c r="F25" s="11"/>
     </row>
     <row r="26" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2" t="s">
+      <c r="A26" s="29"/>
+      <c r="B26" s="29" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="13" t="s">
+      <c r="C26" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="15"/>
+      <c r="D26" s="24"/>
+      <c r="E26" s="24"/>
+      <c r="F26" s="25"/>
     </row>
     <row r="27" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
-      <c r="C27" s="16"/>
-      <c r="D27" s="17"/>
-      <c r="E27" s="17"/>
-      <c r="F27" s="18"/>
+      <c r="A27" s="29"/>
+      <c r="B27" s="29"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="16"/>
     </row>
     <row r="28" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="19" t="s">
+      <c r="A28" s="29"/>
+      <c r="B28" s="29"/>
+      <c r="C28" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="21"/>
+      <c r="D28" s="27"/>
+      <c r="E28" s="27"/>
+      <c r="F28" s="28"/>
     </row>
     <row r="29" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="23"/>
-      <c r="E29" s="23"/>
-      <c r="F29" s="24"/>
+      <c r="A29" s="29"/>
+      <c r="B29" s="29"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="10"/>
+      <c r="E29" s="10"/>
+      <c r="F29" s="11"/>
     </row>
     <row r="30" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2" t="s">
+      <c r="A30" s="29"/>
+      <c r="B30" s="29" t="s">
         <v>11</v>
       </c>
-      <c r="C30" s="13" t="s">
+      <c r="C30" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D30" s="14"/>
-      <c r="E30" s="14"/>
-      <c r="F30" s="15"/>
+      <c r="D30" s="24"/>
+      <c r="E30" s="24"/>
+      <c r="F30" s="25"/>
     </row>
     <row r="31" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="16"/>
-      <c r="D31" s="17"/>
-      <c r="E31" s="17"/>
-      <c r="F31" s="18"/>
+      <c r="A31" s="29"/>
+      <c r="B31" s="29"/>
+      <c r="C31" s="14"/>
+      <c r="D31" s="15"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="16"/>
     </row>
     <row r="32" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
-      <c r="C32" s="19" t="s">
+      <c r="A32" s="29"/>
+      <c r="B32" s="29"/>
+      <c r="C32" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D32" s="20"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="21"/>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="28"/>
     </row>
     <row r="33" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
-      <c r="C33" s="22"/>
-      <c r="D33" s="23"/>
-      <c r="E33" s="23"/>
-      <c r="F33" s="24"/>
+      <c r="A33" s="29"/>
+      <c r="B33" s="29"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="10"/>
+      <c r="E33" s="10"/>
+      <c r="F33" s="11"/>
     </row>
     <row r="34" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2" t="s">
+      <c r="A34" s="29"/>
+      <c r="B34" s="29" t="s">
         <v>10</v>
       </c>
-      <c r="C34" s="13" t="s">
+      <c r="C34" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="15"/>
+      <c r="D34" s="24"/>
+      <c r="E34" s="24"/>
+      <c r="F34" s="25"/>
     </row>
     <row r="35" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
-      <c r="C35" s="16"/>
-      <c r="D35" s="17"/>
-      <c r="E35" s="17"/>
-      <c r="F35" s="18"/>
+      <c r="A35" s="29"/>
+      <c r="B35" s="29"/>
+      <c r="C35" s="14"/>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="16"/>
     </row>
     <row r="36" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="19" t="s">
+      <c r="A36" s="29"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="21"/>
+      <c r="D36" s="27"/>
+      <c r="E36" s="27"/>
+      <c r="F36" s="28"/>
     </row>
     <row r="37" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
-      <c r="C37" s="22"/>
-      <c r="D37" s="23"/>
-      <c r="E37" s="23"/>
-      <c r="F37" s="24"/>
+      <c r="A37" s="29"/>
+      <c r="B37" s="29"/>
+      <c r="C37" s="9"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="10"/>
+      <c r="F37" s="11"/>
     </row>
     <row r="38" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2" t="s">
+      <c r="A38" s="29"/>
+      <c r="B38" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="15"/>
+      <c r="D38" s="24"/>
+      <c r="E38" s="24"/>
+      <c r="F38" s="25"/>
     </row>
     <row r="39" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
-      <c r="C39" s="16"/>
-      <c r="D39" s="17"/>
-      <c r="E39" s="17"/>
-      <c r="F39" s="18"/>
+      <c r="A39" s="29"/>
+      <c r="B39" s="29"/>
+      <c r="C39" s="14"/>
+      <c r="D39" s="15"/>
+      <c r="E39" s="15"/>
+      <c r="F39" s="16"/>
     </row>
     <row r="40" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
-      <c r="C40" s="19" t="s">
+      <c r="A40" s="29"/>
+      <c r="B40" s="29"/>
+      <c r="C40" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="D40" s="20"/>
-      <c r="E40" s="20"/>
-      <c r="F40" s="21"/>
+      <c r="D40" s="27"/>
+      <c r="E40" s="27"/>
+      <c r="F40" s="28"/>
     </row>
     <row r="41" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="22"/>
-      <c r="D41" s="23"/>
-      <c r="E41" s="23"/>
-      <c r="F41" s="24"/>
+      <c r="A41" s="29"/>
+      <c r="B41" s="29"/>
+      <c r="C41" s="9"/>
+      <c r="D41" s="10"/>
+      <c r="E41" s="10"/>
+      <c r="F41" s="11"/>
     </row>
     <row r="42" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="2" t="s">
+      <c r="A42" s="29" t="s">
         <v>13</v>
       </c>
-      <c r="B42" s="2" t="s">
+      <c r="B42" s="29" t="s">
         <v>14</v>
       </c>
-      <c r="C42" s="13" t="s">
+      <c r="C42" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="D42" s="14"/>
-      <c r="E42" s="14"/>
-      <c r="F42" s="15"/>
+      <c r="D42" s="24"/>
+      <c r="E42" s="24"/>
+      <c r="F42" s="25"/>
     </row>
     <row r="43" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="16" t="s">
+      <c r="A43" s="29"/>
+      <c r="B43" s="29"/>
+      <c r="C43" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="D43" s="17"/>
-      <c r="E43" s="17"/>
-      <c r="F43" s="18"/>
+      <c r="D43" s="15"/>
+      <c r="E43" s="15"/>
+      <c r="F43" s="16"/>
     </row>
     <row r="44" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="25"/>
-      <c r="D44" s="26"/>
-      <c r="E44" s="26"/>
-      <c r="F44" s="27"/>
+      <c r="A44" s="29"/>
+      <c r="B44" s="29"/>
+      <c r="C44" s="5"/>
+      <c r="D44" s="6"/>
+      <c r="E44" s="6"/>
+      <c r="F44" s="7"/>
     </row>
     <row r="45" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="16"/>
-      <c r="D45" s="17"/>
-      <c r="E45" s="17"/>
-      <c r="F45" s="18"/>
+      <c r="A45" s="29"/>
+      <c r="B45" s="29"/>
+      <c r="C45" s="14"/>
+      <c r="D45" s="15"/>
+      <c r="E45" s="15"/>
+      <c r="F45" s="16"/>
     </row>
     <row r="46" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="16" t="s">
+      <c r="A46" s="29"/>
+      <c r="B46" s="29"/>
+      <c r="C46" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D46" s="17"/>
-      <c r="E46" s="17"/>
-      <c r="F46" s="18"/>
+      <c r="D46" s="15"/>
+      <c r="E46" s="15"/>
+      <c r="F46" s="16"/>
     </row>
     <row r="47" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A47" s="2"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="16"/>
-      <c r="D47" s="17"/>
-      <c r="E47" s="17"/>
-      <c r="F47" s="18"/>
+      <c r="A47" s="29"/>
+      <c r="B47" s="29"/>
+      <c r="C47" s="14"/>
+      <c r="D47" s="15"/>
+      <c r="E47" s="15"/>
+      <c r="F47" s="16"/>
     </row>
     <row r="48" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A48" s="2"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="16"/>
-      <c r="D48" s="17"/>
-      <c r="E48" s="17"/>
-      <c r="F48" s="18"/>
+      <c r="A48" s="29"/>
+      <c r="B48" s="29"/>
+      <c r="C48" s="14"/>
+      <c r="D48" s="15"/>
+      <c r="E48" s="15"/>
+      <c r="F48" s="16"/>
     </row>
     <row r="49" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A49" s="2"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="28" t="s">
+      <c r="A49" s="29"/>
+      <c r="B49" s="29"/>
+      <c r="C49" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="D49" s="29"/>
-      <c r="E49" s="29"/>
-      <c r="F49" s="30"/>
+      <c r="D49" s="18"/>
+      <c r="E49" s="18"/>
+      <c r="F49" s="19"/>
     </row>
     <row r="50" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A50" s="2"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="16" t="s">
+      <c r="A50" s="29"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="D50" s="17"/>
-      <c r="E50" s="17"/>
-      <c r="F50" s="18"/>
+      <c r="D50" s="15"/>
+      <c r="E50" s="15"/>
+      <c r="F50" s="16"/>
     </row>
     <row r="51" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A51" s="2"/>
-      <c r="B51" s="2"/>
-      <c r="C51" s="16"/>
-      <c r="D51" s="17"/>
-      <c r="E51" s="17"/>
-      <c r="F51" s="18"/>
+      <c r="A51" s="29"/>
+      <c r="B51" s="29"/>
+      <c r="C51" s="14"/>
+      <c r="D51" s="15"/>
+      <c r="E51" s="15"/>
+      <c r="F51" s="16"/>
     </row>
     <row r="52" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="2"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="25"/>
-      <c r="D52" s="26"/>
-      <c r="E52" s="26"/>
-      <c r="F52" s="27"/>
+      <c r="A52" s="29"/>
+      <c r="B52" s="29"/>
+      <c r="C52" s="5"/>
+      <c r="D52" s="6"/>
+      <c r="E52" s="6"/>
+      <c r="F52" s="7"/>
     </row>
     <row r="53" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="2"/>
-      <c r="B53" s="2"/>
-      <c r="C53" s="16" t="s">
+      <c r="A53" s="29"/>
+      <c r="B53" s="29"/>
+      <c r="C53" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="D53" s="17"/>
-      <c r="E53" s="17"/>
-      <c r="F53" s="18"/>
+      <c r="D53" s="15"/>
+      <c r="E53" s="15"/>
+      <c r="F53" s="16"/>
     </row>
     <row r="54" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="16"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="17"/>
-      <c r="F54" s="18"/>
+      <c r="A54" s="29"/>
+      <c r="B54" s="29"/>
+      <c r="C54" s="14"/>
+      <c r="D54" s="15"/>
+      <c r="E54" s="15"/>
+      <c r="F54" s="16"/>
     </row>
     <row r="55" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="2"/>
-      <c r="B55" s="2"/>
-      <c r="C55" s="16"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="17"/>
-      <c r="F55" s="18"/>
+      <c r="A55" s="29"/>
+      <c r="B55" s="29"/>
+      <c r="C55" s="14"/>
+      <c r="D55" s="15"/>
+      <c r="E55" s="15"/>
+      <c r="F55" s="16"/>
     </row>
     <row r="56" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="2"/>
-      <c r="B56" s="2"/>
-      <c r="C56" s="16"/>
-      <c r="D56" s="17"/>
-      <c r="E56" s="17"/>
-      <c r="F56" s="18"/>
+      <c r="A56" s="29"/>
+      <c r="B56" s="29"/>
+      <c r="C56" s="14"/>
+      <c r="D56" s="15"/>
+      <c r="E56" s="15"/>
+      <c r="F56" s="16"/>
     </row>
     <row r="57" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A57" s="2"/>
-      <c r="B57" s="2"/>
-      <c r="C57" s="28" t="s">
+      <c r="A57" s="29"/>
+      <c r="B57" s="29"/>
+      <c r="C57" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="D57" s="29"/>
-      <c r="E57" s="29"/>
-      <c r="F57" s="30"/>
+      <c r="D57" s="18"/>
+      <c r="E57" s="18"/>
+      <c r="F57" s="19"/>
     </row>
     <row r="58" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="2"/>
-      <c r="B58" s="2"/>
-      <c r="C58" s="16"/>
-      <c r="D58" s="17"/>
-      <c r="E58" s="17"/>
-      <c r="F58" s="18"/>
-      <c r="H58" s="11"/>
-      <c r="I58" s="11"/>
-      <c r="J58" s="11"/>
-      <c r="K58" s="11"/>
-      <c r="L58" s="11"/>
-      <c r="M58" s="11"/>
-      <c r="N58" s="11"/>
+      <c r="A58" s="29"/>
+      <c r="B58" s="29"/>
+      <c r="C58" s="14"/>
+      <c r="D58" s="15"/>
+      <c r="E58" s="15"/>
+      <c r="F58" s="16"/>
+      <c r="H58" s="4"/>
+      <c r="I58" s="4"/>
+      <c r="J58" s="4"/>
+      <c r="K58" s="4"/>
+      <c r="L58" s="4"/>
+      <c r="M58" s="4"/>
+      <c r="N58" s="4"/>
     </row>
     <row r="59" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A59" s="2"/>
-      <c r="B59" s="2"/>
-      <c r="C59" s="16"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="17"/>
-      <c r="F59" s="18"/>
-      <c r="H59" s="12"/>
-      <c r="I59" s="12"/>
-      <c r="J59" s="12"/>
-      <c r="K59" s="12"/>
-      <c r="L59" s="12"/>
-      <c r="M59" s="12"/>
-      <c r="N59" s="12"/>
+      <c r="A59" s="29"/>
+      <c r="B59" s="29"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="15"/>
+      <c r="E59" s="15"/>
+      <c r="F59" s="16"/>
+      <c r="H59" s="8"/>
+      <c r="I59" s="8"/>
+      <c r="J59" s="8"/>
+      <c r="K59" s="8"/>
+      <c r="L59" s="8"/>
+      <c r="M59" s="8"/>
+      <c r="N59" s="8"/>
     </row>
     <row r="60" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A60" s="2"/>
-      <c r="B60" s="2"/>
-      <c r="C60" s="16"/>
-      <c r="D60" s="17"/>
-      <c r="E60" s="17"/>
-      <c r="F60" s="18"/>
-      <c r="H60" s="12"/>
-      <c r="I60" s="12"/>
-      <c r="J60" s="12"/>
-      <c r="K60" s="12"/>
-      <c r="L60" s="12"/>
-      <c r="M60" s="12"/>
-      <c r="N60" s="12"/>
+      <c r="A60" s="29"/>
+      <c r="B60" s="29"/>
+      <c r="C60" s="14"/>
+      <c r="D60" s="15"/>
+      <c r="E60" s="15"/>
+      <c r="F60" s="16"/>
+      <c r="H60" s="8"/>
+      <c r="I60" s="8"/>
+      <c r="J60" s="8"/>
+      <c r="K60" s="8"/>
+      <c r="L60" s="8"/>
+      <c r="M60" s="8"/>
+      <c r="N60" s="8"/>
     </row>
     <row r="61" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A61" s="2"/>
-      <c r="B61" s="2"/>
-      <c r="C61" s="16" t="s">
+      <c r="A61" s="29"/>
+      <c r="B61" s="29"/>
+      <c r="C61" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="D61" s="17"/>
-      <c r="E61" s="17"/>
-      <c r="F61" s="18"/>
+      <c r="D61" s="15"/>
+      <c r="E61" s="15"/>
+      <c r="F61" s="16"/>
     </row>
     <row r="62" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="16"/>
-      <c r="D62" s="17"/>
-      <c r="E62" s="17"/>
-      <c r="F62" s="18"/>
+      <c r="A62" s="29"/>
+      <c r="B62" s="29"/>
+      <c r="C62" s="14"/>
+      <c r="D62" s="15"/>
+      <c r="E62" s="15"/>
+      <c r="F62" s="16"/>
     </row>
     <row r="63" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A63" s="2"/>
-      <c r="B63" s="2"/>
-      <c r="C63" s="16"/>
-      <c r="D63" s="17"/>
-      <c r="E63" s="17"/>
-      <c r="F63" s="18"/>
+      <c r="A63" s="29"/>
+      <c r="B63" s="29"/>
+      <c r="C63" s="14"/>
+      <c r="D63" s="15"/>
+      <c r="E63" s="15"/>
+      <c r="F63" s="16"/>
     </row>
     <row r="64" spans="1:14" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A64" s="2"/>
-      <c r="B64" s="2" t="s">
+      <c r="A64" s="29"/>
+      <c r="B64" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="C64" s="13" t="s">
+      <c r="C64" s="23" t="s">
         <v>29</v>
       </c>
-      <c r="D64" s="14"/>
-      <c r="E64" s="14"/>
-      <c r="F64" s="15"/>
+      <c r="D64" s="24"/>
+      <c r="E64" s="24"/>
+      <c r="F64" s="25"/>
     </row>
     <row r="65" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A65" s="2"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="16"/>
-      <c r="D65" s="17"/>
-      <c r="E65" s="17"/>
-      <c r="F65" s="18"/>
+      <c r="A65" s="29"/>
+      <c r="B65" s="29"/>
+      <c r="C65" s="14"/>
+      <c r="D65" s="15"/>
+      <c r="E65" s="15"/>
+      <c r="F65" s="16"/>
     </row>
     <row r="66" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A66" s="2"/>
-      <c r="B66" s="2"/>
-      <c r="C66" s="16"/>
-      <c r="D66" s="17"/>
-      <c r="E66" s="17"/>
-      <c r="F66" s="18"/>
+      <c r="A66" s="29"/>
+      <c r="B66" s="29"/>
+      <c r="C66" s="14"/>
+      <c r="D66" s="15"/>
+      <c r="E66" s="15"/>
+      <c r="F66" s="16"/>
     </row>
     <row r="67" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A67" s="2"/>
-      <c r="B67" s="2"/>
-      <c r="C67" s="19" t="s">
+      <c r="A67" s="29"/>
+      <c r="B67" s="29"/>
+      <c r="C67" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="D67" s="20"/>
-      <c r="E67" s="20"/>
-      <c r="F67" s="21"/>
+      <c r="D67" s="27"/>
+      <c r="E67" s="27"/>
+      <c r="F67" s="28"/>
     </row>
     <row r="68" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A68" s="2"/>
-      <c r="B68" s="2"/>
-      <c r="C68" s="16"/>
-      <c r="D68" s="17"/>
-      <c r="E68" s="17"/>
-      <c r="F68" s="18"/>
+      <c r="A68" s="29"/>
+      <c r="B68" s="29"/>
+      <c r="C68" s="14"/>
+      <c r="D68" s="15"/>
+      <c r="E68" s="15"/>
+      <c r="F68" s="16"/>
     </row>
     <row r="69" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="2"/>
-      <c r="B69" s="2"/>
-      <c r="C69" s="22"/>
-      <c r="D69" s="23"/>
-      <c r="E69" s="23"/>
-      <c r="F69" s="24"/>
+      <c r="A69" s="29"/>
+      <c r="B69" s="29"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="10"/>
+      <c r="E69" s="10"/>
+      <c r="F69" s="11"/>
     </row>
     <row r="70" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="2"/>
-      <c r="B70" s="2" t="s">
+      <c r="A70" s="29"/>
+      <c r="B70" s="29" t="s">
         <v>16</v>
       </c>
-      <c r="C70" s="31"/>
-      <c r="D70" s="32"/>
-      <c r="E70" s="32"/>
-      <c r="F70" s="33"/>
+      <c r="C70" s="20"/>
+      <c r="D70" s="21"/>
+      <c r="E70" s="21"/>
+      <c r="F70" s="22"/>
     </row>
     <row r="71" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="2"/>
-      <c r="B71" s="2"/>
-      <c r="C71" s="16"/>
-      <c r="D71" s="17"/>
-      <c r="E71" s="17"/>
-      <c r="F71" s="18"/>
+      <c r="A71" s="29"/>
+      <c r="B71" s="29"/>
+      <c r="C71" s="14"/>
+      <c r="D71" s="15"/>
+      <c r="E71" s="15"/>
+      <c r="F71" s="16"/>
     </row>
     <row r="72" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A72" s="2"/>
-      <c r="B72" s="2"/>
-      <c r="C72" s="16"/>
-      <c r="D72" s="17"/>
-      <c r="E72" s="17"/>
-      <c r="F72" s="18"/>
+      <c r="A72" s="29"/>
+      <c r="B72" s="29"/>
+      <c r="C72" s="14"/>
+      <c r="D72" s="15"/>
+      <c r="E72" s="15"/>
+      <c r="F72" s="16"/>
     </row>
     <row r="73" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="2"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="16"/>
-      <c r="D73" s="17"/>
-      <c r="E73" s="17"/>
-      <c r="F73" s="18"/>
+      <c r="A73" s="29"/>
+      <c r="B73" s="29"/>
+      <c r="C73" s="14"/>
+      <c r="D73" s="15"/>
+      <c r="E73" s="15"/>
+      <c r="F73" s="16"/>
     </row>
     <row r="74" spans="1:6" ht="16.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A74" s="2"/>
-      <c r="B74" s="2"/>
-      <c r="C74" s="22"/>
-      <c r="D74" s="23"/>
-      <c r="E74" s="23"/>
-      <c r="F74" s="24"/>
+      <c r="A74" s="29"/>
+      <c r="B74" s="29"/>
+      <c r="C74" s="9"/>
+      <c r="D74" s="10"/>
+      <c r="E74" s="10"/>
+      <c r="F74" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="95">
-    <mergeCell ref="N59:N60"/>
-    <mergeCell ref="H59:H60"/>
-    <mergeCell ref="I59:I60"/>
-    <mergeCell ref="J59:J60"/>
-    <mergeCell ref="K59:K60"/>
-    <mergeCell ref="L59:L60"/>
-    <mergeCell ref="M59:M60"/>
+    <mergeCell ref="A6:A41"/>
+    <mergeCell ref="B42:B63"/>
+    <mergeCell ref="B64:B69"/>
+    <mergeCell ref="B70:B74"/>
+    <mergeCell ref="A42:A74"/>
+    <mergeCell ref="B6:B9"/>
+    <mergeCell ref="B10:B13"/>
+    <mergeCell ref="B14:B17"/>
+    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="D1:D4"/>
+    <mergeCell ref="E2:E4"/>
+    <mergeCell ref="F2:F4"/>
+    <mergeCell ref="A1:B4"/>
+    <mergeCell ref="C1:C2"/>
+    <mergeCell ref="C16:F16"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="C12:F12"/>
+    <mergeCell ref="C13:F13"/>
+    <mergeCell ref="C14:F14"/>
+    <mergeCell ref="C15:F15"/>
+    <mergeCell ref="C28:F28"/>
+    <mergeCell ref="C17:F17"/>
+    <mergeCell ref="C18:F18"/>
+    <mergeCell ref="C19:F19"/>
+    <mergeCell ref="C20:F20"/>
+    <mergeCell ref="C21:F21"/>
+    <mergeCell ref="C22:F22"/>
+    <mergeCell ref="C23:F23"/>
+    <mergeCell ref="C24:F24"/>
+    <mergeCell ref="C25:F25"/>
+    <mergeCell ref="C26:F26"/>
+    <mergeCell ref="C27:F27"/>
+    <mergeCell ref="C40:F40"/>
+    <mergeCell ref="C29:F29"/>
+    <mergeCell ref="C30:F30"/>
+    <mergeCell ref="C31:F31"/>
+    <mergeCell ref="C32:F32"/>
+    <mergeCell ref="C33:F33"/>
+    <mergeCell ref="C34:F34"/>
+    <mergeCell ref="C35:F35"/>
+    <mergeCell ref="C36:F36"/>
+    <mergeCell ref="C37:F37"/>
+    <mergeCell ref="C38:F38"/>
+    <mergeCell ref="C39:F39"/>
+    <mergeCell ref="C60:F60"/>
+    <mergeCell ref="C41:F41"/>
+    <mergeCell ref="C42:F42"/>
+    <mergeCell ref="C43:F43"/>
+    <mergeCell ref="C45:F45"/>
+    <mergeCell ref="C46:F46"/>
+    <mergeCell ref="C47:F47"/>
+    <mergeCell ref="C48:F48"/>
+    <mergeCell ref="C49:F49"/>
+    <mergeCell ref="C50:F50"/>
+    <mergeCell ref="C51:F51"/>
+    <mergeCell ref="C53:F53"/>
+    <mergeCell ref="C64:F64"/>
+    <mergeCell ref="C65:F65"/>
+    <mergeCell ref="C66:F66"/>
+    <mergeCell ref="C67:F67"/>
+    <mergeCell ref="C68:F68"/>
     <mergeCell ref="C74:F74"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="C54:F54"/>
@@ -1634,78 +1705,13 @@
     <mergeCell ref="C72:F72"/>
     <mergeCell ref="C73:F73"/>
     <mergeCell ref="C63:F63"/>
-    <mergeCell ref="C64:F64"/>
-    <mergeCell ref="C65:F65"/>
-    <mergeCell ref="C66:F66"/>
-    <mergeCell ref="C67:F67"/>
-    <mergeCell ref="C68:F68"/>
-    <mergeCell ref="C48:F48"/>
-    <mergeCell ref="C49:F49"/>
-    <mergeCell ref="C50:F50"/>
-    <mergeCell ref="C51:F51"/>
-    <mergeCell ref="C53:F53"/>
-    <mergeCell ref="C60:F60"/>
-    <mergeCell ref="C41:F41"/>
-    <mergeCell ref="C42:F42"/>
-    <mergeCell ref="C43:F43"/>
-    <mergeCell ref="C45:F45"/>
-    <mergeCell ref="C46:F46"/>
-    <mergeCell ref="C47:F47"/>
-    <mergeCell ref="C35:F35"/>
-    <mergeCell ref="C36:F36"/>
-    <mergeCell ref="C37:F37"/>
-    <mergeCell ref="C38:F38"/>
-    <mergeCell ref="C39:F39"/>
-    <mergeCell ref="C40:F40"/>
-    <mergeCell ref="C29:F29"/>
-    <mergeCell ref="C30:F30"/>
-    <mergeCell ref="C31:F31"/>
-    <mergeCell ref="C32:F32"/>
-    <mergeCell ref="C33:F33"/>
-    <mergeCell ref="C34:F34"/>
-    <mergeCell ref="C23:F23"/>
-    <mergeCell ref="C24:F24"/>
-    <mergeCell ref="C25:F25"/>
-    <mergeCell ref="C26:F26"/>
-    <mergeCell ref="C27:F27"/>
-    <mergeCell ref="C28:F28"/>
-    <mergeCell ref="C17:F17"/>
-    <mergeCell ref="C18:F18"/>
-    <mergeCell ref="C19:F19"/>
-    <mergeCell ref="C20:F20"/>
-    <mergeCell ref="C21:F21"/>
-    <mergeCell ref="C22:F22"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="C12:F12"/>
-    <mergeCell ref="C13:F13"/>
-    <mergeCell ref="C14:F14"/>
-    <mergeCell ref="C15:F15"/>
-    <mergeCell ref="C16:F16"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C10:F10"/>
-    <mergeCell ref="D1:D4"/>
-    <mergeCell ref="E2:E4"/>
-    <mergeCell ref="F2:F4"/>
-    <mergeCell ref="A1:B4"/>
-    <mergeCell ref="C1:C2"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="A6:A41"/>
-    <mergeCell ref="B42:B63"/>
-    <mergeCell ref="B64:B69"/>
-    <mergeCell ref="B70:B74"/>
-    <mergeCell ref="A42:A74"/>
-    <mergeCell ref="B6:B9"/>
-    <mergeCell ref="B10:B13"/>
-    <mergeCell ref="B14:B17"/>
-    <mergeCell ref="B18:B21"/>
+    <mergeCell ref="N59:N60"/>
+    <mergeCell ref="H59:H60"/>
+    <mergeCell ref="I59:I60"/>
+    <mergeCell ref="J59:J60"/>
+    <mergeCell ref="K59:K60"/>
+    <mergeCell ref="L59:L60"/>
+    <mergeCell ref="M59:M60"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <printOptions horizontalCentered="1"/>

</xml_diff>